<commit_message>
change: move homepage more-info text from hardcoded markdown to config database
</commit_message>
<xml_diff>
--- a/public/data/db-source/config.xlsx
+++ b/public/data/db-source/config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10322"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db_source/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67742504-95B6-2643-8A71-FFB14369FEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7308207E-1960-C54E-89B8-17EB96BA8E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>id</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>closed_data : Closed Data</t>
+  </si>
+  <si>
+    <t>more_info</t>
+  </si>
+  <si>
+    <t>Cette version utilise des données fictives à des fins de démonstration.</t>
   </si>
 </sst>
 </file>
@@ -138,8 +144,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}" name="Tableau1" displayName="Tableau1" ref="A1:B4" totalsRowShown="0">
-  <autoFilter ref="A1:B4" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}" name="Tableau1" displayName="Tableau1" ref="A1:B5" totalsRowShown="0">
+  <autoFilter ref="A1:B5" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{A513F0B6-5730-454E-B160-F273AA355AF9}" name="id"/>
     <tableColumn id="3" xr3:uid="{C6F40ACF-8A8F-094A-9103-5E1A8AABEC96}" name="value" dataCellStyle="Lien hypertexte"/>
@@ -470,11 +476,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -495,17 +501,25 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
change: move homepage more-info text from hardcoded markdown to config database (#106)
* change: move homepage more-info text from hardcoded markdown to config database

* fix: include additional statistical terms in columnCleanNames and columnIcons

* refactor: refine language for clarity in about-main-meta documentation

* release: bump version to 0.18.2 and update dependencies
</commit_message>
<xml_diff>
--- a/public/data/db-source/config.xlsx
+++ b/public/data/db-source/config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10322"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db_source/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bassim/code/datannur/datannur_dev/public/data/db-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67742504-95B6-2643-8A71-FFB14369FEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7308207E-1960-C54E-89B8-17EB96BA8E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>id</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>closed_data : Closed Data</t>
+  </si>
+  <si>
+    <t>more_info</t>
+  </si>
+  <si>
+    <t>Cette version utilise des données fictives à des fins de démonstration.</t>
   </si>
 </sst>
 </file>
@@ -138,8 +144,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}" name="Tableau1" displayName="Tableau1" ref="A1:B4" totalsRowShown="0">
-  <autoFilter ref="A1:B4" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}" name="Tableau1" displayName="Tableau1" ref="A1:B5" totalsRowShown="0">
+  <autoFilter ref="A1:B5" xr:uid="{9BB74F48-D0F4-FA4B-A818-58266F20AB52}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{A513F0B6-5730-454E-B160-F273AA355AF9}" name="id"/>
     <tableColumn id="3" xr3:uid="{C6F40ACF-8A8F-094A-9103-5E1A8AABEC96}" name="value" dataCellStyle="Lien hypertexte"/>
@@ -470,11 +476,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -495,17 +501,25 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>